<commit_message>
decoupled software & paper reproduction CI
</commit_message>
<xml_diff>
--- a/dataset_info.xlsx
+++ b/dataset_info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oguzh\My_Research\tbma\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oguzh\My_Research\FFL_TBMA\experiments_final_corrected\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF01173A-1B2D-4BDE-8910-1B53E1A19BAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7700DB-8C8D-4021-B966-EC307D467DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1200,8 +1200,8 @@
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2" s="1">
-        <v>0</v>
+      <c r="G2">
+        <v>1</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -1226,8 +1226,8 @@
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" s="1">
-        <v>0</v>
+      <c r="G3">
+        <v>1</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -1252,8 +1252,8 @@
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="G4" s="1">
-        <v>0</v>
+      <c r="G4">
+        <v>1</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1281,8 +1281,8 @@
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="G5" s="1">
-        <v>0</v>
+      <c r="G5">
+        <v>1</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1307,8 +1307,8 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="1">
-        <v>0</v>
+      <c r="G6">
+        <v>1</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1336,8 +1336,8 @@
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="G7" s="1">
-        <v>0</v>
+      <c r="G7">
+        <v>1</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1362,8 +1362,8 @@
       <c r="F8">
         <v>0</v>
       </c>
-      <c r="G8" s="1">
-        <v>0</v>
+      <c r="G8">
+        <v>1</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1388,8 +1388,8 @@
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" s="1">
-        <v>0</v>
+      <c r="G9">
+        <v>1</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1443,8 +1443,8 @@
       <c r="F11">
         <v>0</v>
       </c>
-      <c r="G11" s="1">
-        <v>0</v>
+      <c r="G11">
+        <v>1</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1469,8 +1469,8 @@
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="G12" s="1">
-        <v>0</v>
+      <c r="G12">
+        <v>1</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -1576,8 +1576,8 @@
       <c r="F16">
         <v>0</v>
       </c>
-      <c r="G16" s="1">
-        <v>0</v>
+      <c r="G16">
+        <v>1</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1683,8 +1683,8 @@
       <c r="F20">
         <v>0</v>
       </c>
-      <c r="G20" s="1">
-        <v>0</v>
+      <c r="G20">
+        <v>1</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1787,8 +1787,8 @@
       <c r="F24">
         <v>0</v>
       </c>
-      <c r="G24" s="1">
-        <v>0</v>
+      <c r="G24">
+        <v>1</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -2411,8 +2411,8 @@
       <c r="F48">
         <v>0</v>
       </c>
-      <c r="G48" s="1">
-        <v>0</v>
+      <c r="G48">
+        <v>1</v>
       </c>
       <c r="H48">
         <v>1</v>

</xml_diff>